<commit_message>
refactor: update documentation and data structures for Phase 13 - Customer Journey Research
</commit_message>
<xml_diff>
--- a/docs/research/_exports/xlsx/11_Customer_Journey.xlsx
+++ b/docs/research/_exports/xlsx/11_Customer_Journey.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="486">
   <si>
     <t>The 11 Stages Of The Customer Journey</t>
   </si>
@@ -515,10 +515,13 @@
     <t>GOV-018 lists 'incubation unit registration' as a dashboard field. No source documents workflow beyond it.</t>
   </si>
   <si>
-    <t>Incubation Manager / TBI Manager (B-03) is the named role. No source establishes a procurement or spend role for it.</t>
-  </si>
-  <si>
-    <t>Phase 2 documents B-03 and explicitly records its spend authority as UNKNOWN.</t>
+    <t>Incubation Manager / TBI Manager (B-03) is the named role. Phase 2 found no procurement role for it in any source it read.</t>
+  </si>
+  <si>
+    <t>P2-001 is the IIC portal's own guidance on who should be Convener; P2-011 is the named office-holder list. Phase 2 records B-03's procurement role as 'No procurement role found in any source read' and its spend authority as UNKNOWN. The documented absence is the finding.</t>
+  </si>
+  <si>
+    <t>P2-001; P2-011</t>
   </si>
   <si>
     <t>Phase 3B: does the Incubation Manager hold a budget line, and at what ceiling?</t>
@@ -806,10 +809,13 @@
     <t>GOV-027; D1</t>
   </si>
   <si>
-    <t>Startup Activity Coordinator (A-09) implements. Institutional spend authority sits with VC/Director (B-01) and Dean (B-02) at documented ceilings - one of only two Phase 2 roles with DOCUMENTED budget authority.</t>
-  </si>
-  <si>
-    <t>Phase 2 documents the approval chain with named ceilings (NIT Warangal Director = all cases; CRSU VC above Rs 2,00,000; Dean Rs 10,00,000 non-consumable).</t>
+    <t>Startup Activity Coordinator (A-09) implements. Institutional spend authority sits with VC/Director (B-01) and Dean (B-02) at documented ceilings. Four Phase 2 roles carry documented spend authority: B-01, B-02, C-01 (Registrar) and C-03 (Finance Officer).</t>
+  </si>
+  <si>
+    <t>P2-003 (NIT Warangal: Director all cases; Registrar / Dean (R&amp;D) Rs 10,00,000 non-consumable), P2-004 (HoD at Rs 1L, Dean (P&amp;D) at Rs 3L), P2-006 (CRSU: Central Purchase Committee headed by VC above Rs 2 lakhs) and P2-011 (Startup Activity Coordinator = Faculty-in-Charge Incubation Centre) together establish the chain. CORRECTION: the Phase 2 B-01 free-text field says 'one of only two roles', but Phase 2's own grade field records four roles with documented spend authority (B-01, B-02, C-01, C-03). The grade field is used here; the stale prose in data_p2_roles.py line 354 is not.</t>
+  </si>
+  <si>
+    <t>P2-001; P2-003; P2-004; P2-006; P2-011</t>
   </si>
   <si>
     <t>Phase 2 roles A-09, B-01, B-02, C-01, C-03</t>
@@ -3140,13 +3146,13 @@
         <v>78</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>48</v>
+        <v>164</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -3169,10 +3175,10 @@
         <v>91</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>78</v>
@@ -3181,10 +3187,10 @@
         <v>124</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -3207,22 +3213,22 @@
         <v>99</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -3245,22 +3251,22 @@
         <v>107</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K27" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -3283,10 +3289,10 @@
         <v>113</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I28" s="6" t="s">
         <v>102</v>
@@ -3295,10 +3301,10 @@
         <v>48</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="L28" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -3321,22 +3327,22 @@
         <v>75</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K29" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L29" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -3359,10 +3365,10 @@
         <v>83</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I30" s="7" t="s">
         <v>86</v>
@@ -3371,10 +3377,10 @@
         <v>48</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -3397,22 +3403,22 @@
         <v>91</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -3435,10 +3441,10 @@
         <v>99</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I32" s="6" t="s">
         <v>102</v>
@@ -3447,10 +3453,10 @@
         <v>48</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -3473,10 +3479,10 @@
         <v>107</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I33" s="7" t="s">
         <v>86</v>
@@ -3485,10 +3491,10 @@
         <v>48</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -3511,10 +3517,10 @@
         <v>113</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>102</v>
@@ -3523,10 +3529,10 @@
         <v>48</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -3549,22 +3555,22 @@
         <v>75</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K35" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -3587,10 +3593,10 @@
         <v>83</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>78</v>
@@ -3625,10 +3631,10 @@
         <v>91</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>78</v>
@@ -3640,7 +3646,7 @@
         <v>48</v>
       </c>
       <c r="L37" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -3663,16 +3669,16 @@
         <v>99</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K38" s="5" t="s">
         <v>48</v>
@@ -3701,10 +3707,10 @@
         <v>107</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>78</v>
@@ -3716,7 +3722,7 @@
         <v>48</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -3739,22 +3745,22 @@
         <v>113</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -3777,22 +3783,22 @@
         <v>75</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K41" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -3815,22 +3821,22 @@
         <v>83</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="K42" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -3853,22 +3859,22 @@
         <v>91</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K43" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -3891,22 +3897,22 @@
         <v>99</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K44" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -3929,22 +3935,22 @@
         <v>107</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K45" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -3967,22 +3973,22 @@
         <v>113</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K46" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -4005,10 +4011,10 @@
         <v>75</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="I47" s="6" t="s">
         <v>102</v>
@@ -4017,10 +4023,10 @@
         <v>48</v>
       </c>
       <c r="K47" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -4043,10 +4049,10 @@
         <v>83</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I48" s="6" t="s">
         <v>102</v>
@@ -4055,10 +4061,10 @@
         <v>48</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -4081,10 +4087,10 @@
         <v>91</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I49" s="6" t="s">
         <v>102</v>
@@ -4093,10 +4099,10 @@
         <v>48</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -4119,10 +4125,10 @@
         <v>99</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I50" s="6" t="s">
         <v>102</v>
@@ -4131,10 +4137,10 @@
         <v>48</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -4157,10 +4163,10 @@
         <v>107</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I51" s="6" t="s">
         <v>102</v>
@@ -4169,10 +4175,10 @@
         <v>48</v>
       </c>
       <c r="K51" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="L51" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -4195,10 +4201,10 @@
         <v>113</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I52" s="6" t="s">
         <v>102</v>
@@ -4207,10 +4213,10 @@
         <v>48</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -4233,22 +4239,22 @@
         <v>75</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J53" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K53" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L53" s="5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -4271,22 +4277,22 @@
         <v>83</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>48</v>
+        <v>262</v>
       </c>
       <c r="K54" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -4309,22 +4315,22 @@
         <v>91</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J55" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K55" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L55" s="5" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -4347,22 +4353,22 @@
         <v>99</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="I56" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K56" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -4385,22 +4391,22 @@
         <v>107</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="I57" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="K57" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -4423,22 +4429,22 @@
         <v>113</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J58" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K58" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -4461,10 +4467,10 @@
         <v>75</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="I59" s="6" t="s">
         <v>102</v>
@@ -4473,10 +4479,10 @@
         <v>48</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -4499,10 +4505,10 @@
         <v>83</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I60" s="6" t="s">
         <v>102</v>
@@ -4511,10 +4517,10 @@
         <v>48</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="L60" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -4537,10 +4543,10 @@
         <v>91</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I61" s="6" t="s">
         <v>102</v>
@@ -4549,10 +4555,10 @@
         <v>48</v>
       </c>
       <c r="K61" s="5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="L61" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -4575,10 +4581,10 @@
         <v>99</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I62" s="6" t="s">
         <v>102</v>
@@ -4587,10 +4593,10 @@
         <v>48</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -4613,10 +4619,10 @@
         <v>107</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="I63" s="6" t="s">
         <v>102</v>
@@ -4625,10 +4631,10 @@
         <v>48</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -4651,10 +4657,10 @@
         <v>113</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I64" s="6" t="s">
         <v>102</v>
@@ -4663,10 +4669,10 @@
         <v>48</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -4689,22 +4695,22 @@
         <v>75</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="K65" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L65" s="5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -4727,22 +4733,22 @@
         <v>83</v>
       </c>
       <c r="G66" s="5" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="I66" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J66" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="K66" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L66" s="5" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -4765,22 +4771,22 @@
         <v>91</v>
       </c>
       <c r="G67" s="5" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="H67" s="5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="I67" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J67" s="5" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="K67" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L67" s="5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -4803,22 +4809,22 @@
         <v>99</v>
       </c>
       <c r="G68" s="5" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="H68" s="5" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="I68" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="K68" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L68" s="5" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -4841,22 +4847,22 @@
         <v>107</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H69" s="5" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="I69" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J69" s="5" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="K69" s="5" t="s">
         <v>48</v>
       </c>
       <c r="L69" s="5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -4879,22 +4885,22 @@
         <v>113</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H70" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="I70" s="8" t="s">
         <v>78</v>
       </c>
       <c r="J70" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="L70" s="5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -4921,17 +4927,17 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="32" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>63</v>
@@ -4940,13 +4946,13 @@
         <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>69</v>
@@ -4960,7 +4966,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="4" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>18</v>
@@ -4972,10 +4978,10 @@
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>78</v>
@@ -4984,12 +4990,12 @@
         <v>134</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="4" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>18</v>
@@ -5001,10 +5007,10 @@
         <v>3</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>78</v>
@@ -5018,7 +5024,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>37</v>
@@ -5030,10 +5036,10 @@
         <v>3</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>78</v>
@@ -5042,12 +5048,12 @@
         <v>160</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>24</v>
@@ -5059,10 +5065,10 @@
         <v>2</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>78</v>
@@ -5071,12 +5077,12 @@
         <v>148</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="4" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>24</v>
@@ -5088,10 +5094,10 @@
         <v>2</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>78</v>
@@ -5100,12 +5106,12 @@
         <v>155</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="4" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>41</v>
@@ -5117,24 +5123,24 @@
         <v>3</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>78</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="4" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>50</v>
@@ -5146,24 +5152,24 @@
         <v>3</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>78</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="4" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>57</v>
@@ -5175,24 +5181,24 @@
         <v>3</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>78</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="4" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>57</v>
@@ -5204,24 +5210,24 @@
         <v>3</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>78</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="4" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>57</v>
@@ -5233,24 +5239,24 @@
         <v>2</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>78</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="4" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>29</v>
@@ -5262,24 +5268,24 @@
         <v>2</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>78</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="4" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>33</v>
@@ -5291,10 +5297,10 @@
         <v>2</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>86</v>
@@ -5303,12 +5309,12 @@
         <v>48</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>12</v>
@@ -5320,10 +5326,10 @@
         <v>2</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>78</v>
@@ -5337,7 +5343,7 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="4" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>57</v>
@@ -5349,19 +5355,19 @@
         <v>2</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>78</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
   </sheetData>
@@ -5389,17 +5395,17 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="32" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>63</v>
@@ -5408,16 +5414,16 @@
         <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>69</v>
@@ -5431,7 +5437,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>18</v>
@@ -5440,22 +5446,22 @@
         <v>19</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>78</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>131</v>
@@ -5463,7 +5469,7 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>18</v>
@@ -5472,16 +5478,16 @@
         <v>19</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>78</v>
@@ -5495,7 +5501,7 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>18</v>
@@ -5504,16 +5510,16 @@
         <v>19</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>78</v>
@@ -5527,7 +5533,7 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>57</v>
@@ -5536,30 +5542,30 @@
         <v>58</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>78</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>50</v>
@@ -5568,30 +5574,30 @@
         <v>51</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>78</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>57</v>
@@ -5600,30 +5606,30 @@
         <v>58</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>31</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>78</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>57</v>
@@ -5632,16 +5638,16 @@
         <v>58</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>78</v>
@@ -5650,30 +5656,30 @@
         <v>124</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>102</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>102</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>102</v>
@@ -5687,25 +5693,25 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>102</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>102</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>102</v>
@@ -5714,12 +5720,12 @@
         <v>48</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>12</v>
@@ -5731,13 +5737,13 @@
         <v>102</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>102</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>102</v>
@@ -5746,7 +5752,7 @@
         <v>48</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -5770,12 +5776,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
@@ -5892,10 +5898,10 @@
         <v>102</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -5912,10 +5918,10 @@
         <v>86</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -5932,10 +5938,10 @@
         <v>102</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -5952,10 +5958,10 @@
         <v>86</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -5972,10 +5978,10 @@
         <v>102</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -5992,10 +5998,10 @@
         <v>102</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -6012,10 +6018,10 @@
         <v>102</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -6032,10 +6038,10 @@
         <v>102</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -6052,10 +6058,10 @@
         <v>102</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -6072,10 +6078,10 @@
         <v>102</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -6092,10 +6098,10 @@
         <v>102</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -6112,10 +6118,10 @@
         <v>102</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -6132,10 +6138,10 @@
         <v>102</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -6152,10 +6158,10 @@
         <v>102</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -6172,10 +6178,10 @@
         <v>102</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -6192,10 +6198,10 @@
         <v>102</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -6212,27 +6218,27 @@
         <v>102</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>102</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>117</v>
@@ -6240,22 +6246,22 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>102</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -6266,16 +6272,16 @@
         <v>13</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>102</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -6299,23 +6305,23 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>69</v>
@@ -6324,247 +6330,247 @@
         <v>70</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="4" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="4" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="4" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="4" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>